<commit_message>
Adjust leger export formatting
</commit_message>
<xml_diff>
--- a/public/template/template-leger.xlsx
+++ b/public/template/template-leger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/XAMPP/xamppfiles/htdocs/sianida/public/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30269D71-2E57-404C-A3A9-B857123BA6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2962CF8A-3103-CA42-B178-65D380CDAAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t>Sekolah</t>
   </si>
@@ -59,9 +59,6 @@
   </si>
   <si>
     <t>: 20328970</t>
-  </si>
-  <si>
-    <t>Semester</t>
   </si>
   <si>
     <t>: {{ semester_terpilih }}</t>
@@ -518,7 +515,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="8"/>
     </row>
@@ -528,17 +525,13 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>9</v>
-      </c>
+      <c r="A5" s="7"/>
       <c r="B5" s="7"/>
-      <c r="C5" s="7" t="s">
-        <v>10</v>
-      </c>
+      <c r="C5" s="7"/>
       <c r="D5" s="7"/>
     </row>
     <row r="7" spans="1:6" ht="50" customHeight="1" x14ac:dyDescent="0.2">
@@ -552,13 +545,13 @@
         <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -566,19 +559,19 @@
         <v>1</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -586,19 +579,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -606,19 +599,19 @@
         <v>3</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>